<commit_message>
refactor: score_type verwijderd uit alle configuratiebestanden
Config kolommen-tabblad heeft nu 4 kolommen in plaats van 5:
kolom_naam, instrument, item, criterium (optioneel).

Alle config-bestanden opnieuw gegenereerd:
- config_FAR_Leiden_2025.xlsx
- config_FAR_Leiden_2026.xlsx
- config_Psychologie_2021_2022.xlsx
- config_Psychologie_2022_2023.xlsx
- config_Psychologie_2026_2027.xlsx
- config_template.xlsx
- config_BioMed_AUMC_2026.xlsx (fictief)

Scripts aangepast: update_configs.py, maak_template.py,
maak_fictief_programma.py.
</commit_message>
<xml_diff>
--- a/config_FAR_Leiden_2025.xlsx
+++ b/config_FAR_Leiden_2025.xlsx
@@ -547,14 +547,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="25" customWidth="1" min="2" max="2"/>
     <col width="35" customWidth="1" min="3" max="3"/>
     <col width="25" customWidth="1" min="4" max="4"/>
-    <col width="20" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -578,11 +577,6 @@
           <t>criterium (optioneel)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>score_type</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="4" t="inlineStr">
@@ -605,11 +599,6 @@
           <t>Studieresultaat</t>
         </is>
       </c>
-      <c r="E2" s="4" t="inlineStr">
-        <is>
-          <t>cijfer (1-10)</t>
-        </is>
-      </c>
     </row>
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
@@ -632,11 +621,6 @@
           <t>Studieresultaat</t>
         </is>
       </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>punten</t>
-        </is>
-      </c>
     </row>
     <row r="4">
       <c r="A4" s="4" t="inlineStr">
@@ -659,11 +643,6 @@
           <t>Studietempo</t>
         </is>
       </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>punten</t>
-        </is>
-      </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -686,11 +665,6 @@
           <t>Taalbeheersing</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
-        <is>
-          <t>punten</t>
-        </is>
-      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
@@ -713,11 +687,6 @@
           <t>Taalbeheersing</t>
         </is>
       </c>
-      <c r="E6" s="4" t="inlineStr">
-        <is>
-          <t>punten</t>
-        </is>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -740,11 +709,6 @@
           <t>Taalbeheersing</t>
         </is>
       </c>
-      <c r="E7" s="4" t="inlineStr">
-        <is>
-          <t>punten</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
@@ -767,11 +731,6 @@
           <t>Taalbeheersing</t>
         </is>
       </c>
-      <c r="E8" s="4" t="inlineStr">
-        <is>
-          <t>punten</t>
-        </is>
-      </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
@@ -794,11 +753,6 @@
           <t>Communicatievaardigheid</t>
         </is>
       </c>
-      <c r="E9" s="4" t="inlineStr">
-        <is>
-          <t>punten</t>
-        </is>
-      </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
@@ -821,11 +775,6 @@
           <t>Communicatievaardigheid</t>
         </is>
       </c>
-      <c r="E10" s="4" t="inlineStr">
-        <is>
-          <t>punten</t>
-        </is>
-      </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -844,11 +793,6 @@
         </is>
       </c>
       <c r="D11" s="4" t="inlineStr"/>
-      <c r="E11" s="4" t="inlineStr">
-        <is>
-          <t>punten</t>
-        </is>
-      </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
@@ -867,11 +811,6 @@
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr"/>
-      <c r="E12" s="4" t="inlineStr">
-        <is>
-          <t>punten</t>
-        </is>
-      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>